<commit_message>
Finished all Localization test cases and their implementation
</commit_message>
<xml_diff>
--- a/E-Commerce Web/Amazon/Test Suites/Additional Tables.xlsx
+++ b/E-Commerce Web/Amazon/Test Suites/Additional Tables.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="39" uniqueCount="39">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="42" uniqueCount="42">
   <si>
     <t>Date Format</t>
   </si>
@@ -136,6 +136,15 @@
   </si>
   <si>
     <t>AUD</t>
+  </si>
+  <si>
+    <t>1133.99</t>
+  </si>
+  <si>
+    <t>988.78</t>
+  </si>
+  <si>
+    <t>91569.69</t>
   </si>
 </sst>
 </file>
@@ -186,7 +195,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
@@ -211,6 +220,10 @@
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
   </cellXfs>
@@ -493,7 +506,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:J10"/>
+  <dimension ref="A1:J13"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="19.109375" customWidth="1"/>
@@ -645,6 +658,23 @@
         <v>38</v>
       </c>
     </row>
+    <row r="11" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="B11" s="10" t="s">
+        <v>39</v>
+      </c>
+      <c r="C11" t="s">
+        <v>40</v>
+      </c>
+      <c r="D11" s="11" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="12" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="B12" s="10"/>
+    </row>
+    <row r="13" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="B13" s="10"/>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Test Cases and implementation of Exploratory Testing
</commit_message>
<xml_diff>
--- a/E-Commerce Web/Amazon/Test Suites/Additional Tables.xlsx
+++ b/E-Commerce Web/Amazon/Test Suites/Additional Tables.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="42" uniqueCount="42">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="43" uniqueCount="43">
   <si>
     <t>Date Format</t>
   </si>
@@ -145,6 +145,9 @@
   </si>
   <si>
     <t>91569.69</t>
+  </si>
+  <si>
+    <t>TC-EXP-1</t>
   </si>
 </sst>
 </file>
@@ -241,6 +244,49 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>1</xdr:colOff>
+      <xdr:row>18</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>1981201</xdr:colOff>
+      <xdr:row>28</xdr:row>
+      <xdr:rowOff>16199</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="2" name="Рисунок 1"/>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="1" y="4084320"/>
+          <a:ext cx="4198620" cy="1844999"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -506,7 +552,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:J13"/>
+  <dimension ref="A1:J18"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="19.109375" customWidth="1"/>
@@ -675,7 +721,13 @@
     <row r="13" spans="1:10" x14ac:dyDescent="0.3">
       <c r="B13" s="10"/>
     </row>
+    <row r="18" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A18" t="s">
+        <v>42</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Creating Bug Report and Test Summary Report Templates
</commit_message>
<xml_diff>
--- a/E-Commerce Web/Amazon/Test Suites/Additional Tables.xlsx
+++ b/E-Commerce Web/Amazon/Test Suites/Additional Tables.xlsx
@@ -257,9 +257,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>2</xdr:col>
-      <xdr:colOff>1981201</xdr:colOff>
-      <xdr:row>28</xdr:row>
-      <xdr:rowOff>16199</xdr:rowOff>
+      <xdr:colOff>1348741</xdr:colOff>
+      <xdr:row>26</xdr:row>
+      <xdr:rowOff>104037</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -277,7 +277,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="1" y="4084320"/>
-          <a:ext cx="4198620" cy="1844999"/>
+          <a:ext cx="3566160" cy="1567077"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>

</xml_diff>

<commit_message>
Finished Bug Reporting Process
</commit_message>
<xml_diff>
--- a/E-Commerce Web/Amazon/Test Suites/Additional Tables.xlsx
+++ b/E-Commerce Web/Amazon/Test Suites/Additional Tables.xlsx
@@ -251,15 +251,15 @@
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
       <xdr:col>0</xdr:col>
-      <xdr:colOff>1</xdr:colOff>
+      <xdr:colOff>0</xdr:colOff>
       <xdr:row>18</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>2</xdr:col>
-      <xdr:colOff>1348741</xdr:colOff>
-      <xdr:row>26</xdr:row>
-      <xdr:rowOff>104037</xdr:rowOff>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>472439</xdr:colOff>
+      <xdr:row>37</xdr:row>
+      <xdr:rowOff>124869</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -276,8 +276,8 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="1" y="4084320"/>
-          <a:ext cx="3566160" cy="1567077"/>
+          <a:off x="0" y="4084320"/>
+          <a:ext cx="8191499" cy="3599589"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>

</xml_diff>